<commit_message>
Add BC translation scripts
</commit_message>
<xml_diff>
--- a/lookupTables/behavior.xlsx
+++ b/lookupTables/behavior.xlsx
@@ -1,21 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\MelinaStuff\BAM\WildTrax\WT-Integration\lookupTables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A49EA16-EAF2-4295-AEBD-A1A8B1549FE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D925C5A-F392-48EF-B2EA-E3A258C6F412}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
-    <sheet name="Feuil2" sheetId="2" r:id="rId2"/>
+    <sheet name="atlas_breeding_code" sheetId="3" r:id="rId2"/>
+    <sheet name="Feuil2" sheetId="2" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">atlas_breeding_code!$A$1:$M$31</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -36,8 +40,80 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={438F1965-7B7D-477E-A40E-6D281371EABA}</author>
+    <author>tc={D16F95F0-2AF1-4A18-A676-37C91F0DD470}</author>
+    <author>tc={20BEDC8F-E244-44C5-85E0-B6528BA29348}</author>
+    <author>tc={7A719BB3-3A78-4AEA-9227-FFB50AF39344}</author>
+    <author>tc={5C1CCE8D-A372-43D2-BC43-5372A61CACCA}</author>
+    <author>tc={29674C56-20D9-4262-BC3F-68E41BF8DEA1}</author>
+    <author>tc={A3DA788C-BC7D-4061-8AEB-90A0AB7E4085}</author>
+  </authors>
+  <commentList>
+    <comment ref="F1" authorId="0" shapeId="0" xr:uid="{438F1965-7B7D-477E-A40E-6D281371EABA}">
+      <text>
+        <t>[Commentaire à thread]
+Votre version d’Excel vous permet de lire ce commentaire à thread. Toutefois, les modifications qui y sont apportées seront supprimées si le fichier est ouvert dans une version plus récente d’Excel. En savoir plus : https://go.microsoft.com/fwlink/?linkid=870924
+Commentaire :
+    Song / Calls / Flight calls / Non-vocal / DNC</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="1" shapeId="0" xr:uid="{D16F95F0-2AF1-4A18-A676-37C91F0DD470}">
+      <text>
+        <t>[Commentaire à thread]
+Votre version d’Excel vous permet de lire ce commentaire à thread. Toutefois, les modifications qui y sont apportées seront supprimées si le fichier est ouvert dans une version plus récente d’Excel. En savoir plus : https://go.microsoft.com/fwlink/?linkid=870924
+Commentaire :
+    Drumming, counter-singing, ...</t>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="2" shapeId="0" xr:uid="{20BEDC8F-E244-44C5-85E0-B6528BA29348}">
+      <text>
+        <t>[Commentaire à thread]
+Votre version d’Excel vous permet de lire ce commentaire à thread. Toutefois, les modifications qui y sont apportées seront supprimées si le fichier est ouvert dans une version plus récente d’Excel. En savoir plus : https://go.microsoft.com/fwlink/?linkid=870924
+Commentaire :
+    Adult / Juvenile / Fledgking / Immature</t>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="3" shapeId="0" xr:uid="{7A719BB3-3A78-4AEA-9227-FFB50AF39344}">
+      <text>
+        <t>[Commentaire à thread]
+Votre version d’Excel vous permet de lire ce commentaire à thread. Toutefois, les modifications qui y sont apportées seront supprimées si le fichier est ouvert dans une version plus récente d’Excel. En savoir plus : https://go.microsoft.com/fwlink/?linkid=870924
+Commentaire :
+    Male / Female</t>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="4" shapeId="0" xr:uid="{5C1CCE8D-A372-43D2-BC43-5372A61CACCA}">
+      <text>
+        <t>[Commentaire à thread]
+Votre version d’Excel vous permet de lire ce commentaire à thread. Toutefois, les modifications qui y sont apportées seront supprimées si le fichier est ouvert dans une version plus récente d’Excel. En savoir plus : https://go.microsoft.com/fwlink/?linkid=870924
+Commentaire :
+    Flock /Pair / Family group</t>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="5" shapeId="0" xr:uid="{29674C56-20D9-4262-BC3F-68E41BF8DEA1}">
+      <text>
+        <t>[Commentaire à thread]
+Votre version d’Excel vous permet de lire ce commentaire à thread. Toutefois, les modifications qui y sont apportées seront supprimées si le fichier est ouvert dans une version plus récente d’Excel. En savoir plus : https://go.microsoft.com/fwlink/?linkid=870924
+Commentaire :
+    Yes / No</t>
+      </text>
+    </comment>
+    <comment ref="L1" authorId="6" shapeId="0" xr:uid="{A3DA788C-BC7D-4061-8AEB-90A0AB7E4085}">
+      <text>
+        <t>[Commentaire à thread]
+Votre version d’Excel vous permet de lire ce commentaire à thread. Toutefois, les modifications qui y sont apportées seront supprimées si le fichier est ouvert dans une version plus récente d’Excel. En savoir plus : https://go.microsoft.com/fwlink/?linkid=870924
+Commentaire :
+    Aerial display, ...</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="677" uniqueCount="148">
   <si>
     <t>BEHAVIOURID</t>
   </si>
@@ -277,6 +353,210 @@
   </si>
   <si>
     <t>Male / Female</t>
+  </si>
+  <si>
+    <t>Code X (Species observed),</t>
+  </si>
+  <si>
+    <t>Breeding behaviour involving a male and female (e.g., display, courtship feeding and copulation) or antagonistic behaviour between two or more individuals (e.g., territorial disputes or chases), in suitable nesting habitat during the species' breeding season.</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>Nest building, including the carrying of nesting material, by all species except wrens and woodpeckers.</t>
+  </si>
+  <si>
+    <t>CN</t>
+  </si>
+  <si>
+    <t>DD</t>
+  </si>
+  <si>
+    <t>NU</t>
+  </si>
+  <si>
+    <t>Recently fledged (nidicolous species) or downy (nidifugous species) young incapable of sustained flight.</t>
+  </si>
+  <si>
+    <t>JE</t>
+  </si>
+  <si>
+    <t>NO</t>
+  </si>
+  <si>
+    <t>Adult occupying, leaving or entering a probable nest site (visible or not) and whose behaviour suggests the presence of an occupied nest.</t>
+  </si>
+  <si>
+    <t>FE</t>
+  </si>
+  <si>
+    <t>Adult carrying a fecal sac.</t>
+  </si>
+  <si>
+    <t>AT</t>
+  </si>
+  <si>
+    <t>Adult carrying food for young.</t>
+  </si>
+  <si>
+    <t>Nest containing one or more eggs.</t>
+  </si>
+  <si>
+    <t>NF</t>
+  </si>
+  <si>
+    <t>Nest with one or more young (seen or heard).</t>
+  </si>
+  <si>
+    <t>NJ</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>P</t>
+  </si>
+  <si>
+    <t>S</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C </t>
+  </si>
+  <si>
+    <t>V</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>CF</t>
+  </si>
+  <si>
+    <t>CS</t>
+  </si>
+  <si>
+    <t>Adult</t>
+  </si>
+  <si>
+    <t>NB</t>
+  </si>
+  <si>
+    <t>Species observed in its breeding season (no breeding evidence)</t>
+  </si>
+  <si>
+    <t>H</t>
+  </si>
+  <si>
+    <t>Species observed in its breeding season in suitable nesting habitat</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 	Singing male(s) present, or breeding calls heard, in suitable nesting habitat in breeding season</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 	At least 7 individuals singing or producing other sounds associated with breeding (e.g., calls or drumming), heard during the same visit to a single square and in suitable nesting habitat during the species' breeding season.</t>
+  </si>
+  <si>
+    <t>Pair observed in suitable nesting habitat in nesting season</t>
+  </si>
+  <si>
+    <t>T</t>
+  </si>
+  <si>
+    <t>Permanent territory presumed through registration of territorial song, or the occurrence of an adult bird, at the same place, in breeding habitat, on at least two days a week or more apart, during its breeding season. Use discretion when using this code.</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>Courtship or display, including interaction between a male and a female or two males, including courtship feeding or copulation.</t>
+  </si>
+  <si>
+    <t>Visiting probable nest site</t>
+  </si>
+  <si>
+    <t>Agitated behaviour or anxiety calls of an adult</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	Brood Patch on adult female or cloacal protuberance on adult male</t>
+  </si>
+  <si>
+    <t>Nest-building or excavation of nest hole by a wren or a woodpecker</t>
+  </si>
+  <si>
+    <t>Nest-building or excavation of nest hole by a species other than a wren or a woodpecker</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	Distraction display or injury feigning</t>
+  </si>
+  <si>
+    <t>Used nest or egg shells found (occupied or laid within the period of the survey)</t>
+  </si>
+  <si>
+    <t>FY</t>
+  </si>
+  <si>
+    <t>Recently fledged young (nidicolous species) or downy yound (nidifugous species) incapable of sustained flight</t>
+  </si>
+  <si>
+    <t>AE</t>
+  </si>
+  <si>
+    <t>Adult leaving or entering nest sites in circumstances indicating occupied nest</t>
+  </si>
+  <si>
+    <t>FS</t>
+  </si>
+  <si>
+    <t>Adult carying fecal sac</t>
+  </si>
+  <si>
+    <t>Adult carying food for young</t>
+  </si>
+  <si>
+    <t>NE</t>
+  </si>
+  <si>
+    <t>Nest containing eggs</t>
+  </si>
+  <si>
+    <t>NY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	Nest with young seen or heard</t>
+  </si>
+  <si>
+    <t>Counter-singing, counter-calling, other male to male vocal interaction (BAM code)</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Not Applicable</t>
+  </si>
+  <si>
+    <t>Song / Call</t>
+  </si>
+  <si>
+    <t>Courtship</t>
+  </si>
+  <si>
+    <t>Fledging</t>
+  </si>
+  <si>
+    <t>counter-singing</t>
+  </si>
+  <si>
+    <t>Flock</t>
   </si>
 </sst>
 </file>
@@ -286,7 +566,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.00000"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -318,8 +598,39 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color indexed="8"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color indexed="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -338,8 +649,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="22"/>
+        <bgColor indexed="0"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -362,11 +679,42 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="8"/>
+      </left>
+      <right style="thin">
+        <color indexed="8"/>
+      </right>
+      <top style="thin">
+        <color indexed="8"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="8"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="22"/>
+      </left>
+      <right style="thin">
+        <color indexed="22"/>
+      </right>
+      <top style="thin">
+        <color indexed="22"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="22"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -384,9 +732,18 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal_atlas_breeding_code" xfId="1" xr:uid="{288A453B-E530-4E12-B6C1-10A1DB301A4F}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -399,6 +756,12 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Mélina Houle" id="{0858014D-26AE-4040-A589-AC0DB958518C}" userId="S::MEHOU10@ulaval.ca::0e41cf70-ea34-4710-9887-0372e4991b6a" providerId="AD"/>
+</personList>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -716,6 +1079,32 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="F1" dT="2025-04-02T15:38:19.89" personId="{0858014D-26AE-4040-A589-AC0DB958518C}" id="{438F1965-7B7D-477E-A40E-6D281371EABA}">
+    <text>Song / Calls / Flight calls / Non-vocal / DNC</text>
+  </threadedComment>
+  <threadedComment ref="G1" dT="2025-04-02T15:39:04.36" personId="{0858014D-26AE-4040-A589-AC0DB958518C}" id="{D16F95F0-2AF1-4A18-A676-37C91F0DD470}">
+    <text>Drumming, counter-singing, ...</text>
+  </threadedComment>
+  <threadedComment ref="H1" dT="2025-04-02T15:39:20.61" personId="{0858014D-26AE-4040-A589-AC0DB958518C}" id="{20BEDC8F-E244-44C5-85E0-B6528BA29348}">
+    <text>Adult / Juvenile / Fledgking / Immature</text>
+  </threadedComment>
+  <threadedComment ref="I1" dT="2025-04-02T15:39:33.70" personId="{0858014D-26AE-4040-A589-AC0DB958518C}" id="{7A719BB3-3A78-4AEA-9227-FFB50AF39344}">
+    <text>Male / Female</text>
+  </threadedComment>
+  <threadedComment ref="J1" dT="2025-04-02T15:39:48.11" personId="{0858014D-26AE-4040-A589-AC0DB958518C}" id="{5C1CCE8D-A372-43D2-BC43-5372A61CACCA}">
+    <text>Flock /Pair / Family group</text>
+  </threadedComment>
+  <threadedComment ref="K1" dT="2025-04-02T15:39:58.98" personId="{0858014D-26AE-4040-A589-AC0DB958518C}" id="{29674C56-20D9-4262-BC3F-68E41BF8DEA1}">
+    <text>Yes / No</text>
+  </threadedComment>
+  <threadedComment ref="L1" dT="2025-04-02T15:40:21.73" personId="{0858014D-26AE-4040-A589-AC0DB958518C}" id="{A3DA788C-BC7D-4061-8AEB-90A0AB7E4085}">
+    <text>Aerial display, ...</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:N31"/>
@@ -864,7 +1253,9 @@
       <c r="B11" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="C11" s="6"/>
+      <c r="C11" s="6" t="s">
+        <v>80</v>
+      </c>
       <c r="D11" s="6" t="s">
         <v>72</v>
       </c>
@@ -1565,6 +1956,1289 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{928F2DD2-5FFA-4840-99B4-B7403ECB3D45}">
+  <dimension ref="A1:M31"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="109.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A2" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>112</v>
+      </c>
+      <c r="C2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J2" t="s">
+        <v>17</v>
+      </c>
+      <c r="K2" t="s">
+        <v>107</v>
+      </c>
+      <c r="L2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M2" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A3" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="C3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" t="s">
+        <v>17</v>
+      </c>
+      <c r="H3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I3" t="s">
+        <v>17</v>
+      </c>
+      <c r="J3" t="s">
+        <v>17</v>
+      </c>
+      <c r="K3" t="s">
+        <v>107</v>
+      </c>
+      <c r="L3" t="s">
+        <v>17</v>
+      </c>
+      <c r="M3" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A4" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>115</v>
+      </c>
+      <c r="C4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F4" t="s">
+        <v>143</v>
+      </c>
+      <c r="G4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I4" t="s">
+        <v>17</v>
+      </c>
+      <c r="J4" t="s">
+        <v>17</v>
+      </c>
+      <c r="K4" t="s">
+        <v>107</v>
+      </c>
+      <c r="L4" t="s">
+        <v>17</v>
+      </c>
+      <c r="M4" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" s="12" t="s">
+        <v>103</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" t="s">
+        <v>16</v>
+      </c>
+      <c r="E5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F5" t="s">
+        <v>143</v>
+      </c>
+      <c r="G5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I5" t="s">
+        <v>17</v>
+      </c>
+      <c r="J5" t="s">
+        <v>147</v>
+      </c>
+      <c r="K5" t="s">
+        <v>107</v>
+      </c>
+      <c r="L5" t="s">
+        <v>17</v>
+      </c>
+      <c r="M5" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A6" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>117</v>
+      </c>
+      <c r="C6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6" t="s">
+        <v>17</v>
+      </c>
+      <c r="E6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F6" t="s">
+        <v>17</v>
+      </c>
+      <c r="G6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H6" t="s">
+        <v>110</v>
+      </c>
+      <c r="J6" t="s">
+        <v>36</v>
+      </c>
+      <c r="K6" t="s">
+        <v>107</v>
+      </c>
+      <c r="L6" t="s">
+        <v>17</v>
+      </c>
+      <c r="M6" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" ht="45" x14ac:dyDescent="0.25">
+      <c r="A7" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>119</v>
+      </c>
+      <c r="C7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7" t="s">
+        <v>17</v>
+      </c>
+      <c r="F7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G7" t="s">
+        <v>17</v>
+      </c>
+      <c r="H7" t="s">
+        <v>110</v>
+      </c>
+      <c r="I7" t="s">
+        <v>17</v>
+      </c>
+      <c r="J7" t="s">
+        <v>17</v>
+      </c>
+      <c r="K7" t="s">
+        <v>107</v>
+      </c>
+      <c r="L7" t="s">
+        <v>17</v>
+      </c>
+      <c r="M7" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A8" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="C8" t="s">
+        <v>16</v>
+      </c>
+      <c r="D8" t="s">
+        <v>17</v>
+      </c>
+      <c r="E8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F8" t="s">
+        <v>17</v>
+      </c>
+      <c r="G8" t="s">
+        <v>17</v>
+      </c>
+      <c r="H8" t="s">
+        <v>110</v>
+      </c>
+      <c r="I8" t="s">
+        <v>17</v>
+      </c>
+      <c r="J8" t="s">
+        <v>36</v>
+      </c>
+      <c r="K8" t="s">
+        <v>107</v>
+      </c>
+      <c r="L8" t="s">
+        <v>144</v>
+      </c>
+      <c r="M8" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>121</v>
+      </c>
+      <c r="C9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" t="s">
+        <v>17</v>
+      </c>
+      <c r="E9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F9" t="s">
+        <v>17</v>
+      </c>
+      <c r="G9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H9" t="s">
+        <v>110</v>
+      </c>
+      <c r="I9" t="s">
+        <v>17</v>
+      </c>
+      <c r="J9" t="s">
+        <v>36</v>
+      </c>
+      <c r="K9" t="s">
+        <v>107</v>
+      </c>
+      <c r="L9" t="s">
+        <v>144</v>
+      </c>
+      <c r="M9" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A10" s="12" t="s">
+        <v>105</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>122</v>
+      </c>
+      <c r="C10" t="s">
+        <v>16</v>
+      </c>
+      <c r="D10" t="s">
+        <v>17</v>
+      </c>
+      <c r="E10" t="s">
+        <v>16</v>
+      </c>
+      <c r="F10" t="s">
+        <v>17</v>
+      </c>
+      <c r="G10" t="s">
+        <v>17</v>
+      </c>
+      <c r="H10" t="s">
+        <v>110</v>
+      </c>
+      <c r="I10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J10" t="s">
+        <v>17</v>
+      </c>
+      <c r="K10" t="s">
+        <v>107</v>
+      </c>
+      <c r="L10" t="s">
+        <v>17</v>
+      </c>
+      <c r="M10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A11" s="12" t="s">
+        <v>99</v>
+      </c>
+      <c r="B11" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="C11" t="s">
+        <v>16</v>
+      </c>
+      <c r="D11" t="s">
+        <v>16</v>
+      </c>
+      <c r="E11" t="s">
+        <v>16</v>
+      </c>
+      <c r="F11" t="s">
+        <v>18</v>
+      </c>
+      <c r="G11" t="s">
+        <v>17</v>
+      </c>
+      <c r="H11" t="s">
+        <v>110</v>
+      </c>
+      <c r="I11" t="s">
+        <v>17</v>
+      </c>
+      <c r="J11" t="s">
+        <v>17</v>
+      </c>
+      <c r="K11" t="s">
+        <v>107</v>
+      </c>
+      <c r="L11" t="s">
+        <v>17</v>
+      </c>
+      <c r="M11" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A12" s="12" t="s">
+        <v>106</v>
+      </c>
+      <c r="B12" s="12" t="s">
+        <v>124</v>
+      </c>
+      <c r="C12" t="s">
+        <v>16</v>
+      </c>
+      <c r="D12" t="s">
+        <v>17</v>
+      </c>
+      <c r="E12" t="s">
+        <v>16</v>
+      </c>
+      <c r="F12" t="s">
+        <v>17</v>
+      </c>
+      <c r="G12" t="s">
+        <v>17</v>
+      </c>
+      <c r="H12" t="s">
+        <v>110</v>
+      </c>
+      <c r="I12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J12" t="s">
+        <v>17</v>
+      </c>
+      <c r="K12" t="s">
+        <v>107</v>
+      </c>
+      <c r="L12" t="s">
+        <v>17</v>
+      </c>
+      <c r="M12" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A13" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="B13" s="12" t="s">
+        <v>125</v>
+      </c>
+      <c r="C13" t="s">
+        <v>16</v>
+      </c>
+      <c r="D13" t="s">
+        <v>17</v>
+      </c>
+      <c r="E13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F13" t="s">
+        <v>17</v>
+      </c>
+      <c r="G13" t="s">
+        <v>17</v>
+      </c>
+      <c r="H13" t="s">
+        <v>110</v>
+      </c>
+      <c r="I13" t="s">
+        <v>17</v>
+      </c>
+      <c r="J13" t="s">
+        <v>17</v>
+      </c>
+      <c r="K13" t="s">
+        <v>107</v>
+      </c>
+      <c r="L13" t="s">
+        <v>17</v>
+      </c>
+      <c r="M13" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A14" s="12" t="s">
+        <v>111</v>
+      </c>
+      <c r="B14" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="C14" t="s">
+        <v>16</v>
+      </c>
+      <c r="D14" t="s">
+        <v>17</v>
+      </c>
+      <c r="E14" t="s">
+        <v>16</v>
+      </c>
+      <c r="F14" t="s">
+        <v>17</v>
+      </c>
+      <c r="G14" t="s">
+        <v>17</v>
+      </c>
+      <c r="H14" t="s">
+        <v>110</v>
+      </c>
+      <c r="I14" t="s">
+        <v>17</v>
+      </c>
+      <c r="J14" t="s">
+        <v>17</v>
+      </c>
+      <c r="K14" t="s">
+        <v>107</v>
+      </c>
+      <c r="L14" t="s">
+        <v>17</v>
+      </c>
+      <c r="M14" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A15" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="B15" s="12" t="s">
+        <v>127</v>
+      </c>
+      <c r="C15" t="s">
+        <v>16</v>
+      </c>
+      <c r="D15" t="s">
+        <v>17</v>
+      </c>
+      <c r="E15" t="s">
+        <v>16</v>
+      </c>
+      <c r="F15" t="s">
+        <v>17</v>
+      </c>
+      <c r="G15" t="s">
+        <v>17</v>
+      </c>
+      <c r="H15" t="s">
+        <v>110</v>
+      </c>
+      <c r="I15" t="s">
+        <v>17</v>
+      </c>
+      <c r="J15" t="s">
+        <v>17</v>
+      </c>
+      <c r="K15" t="s">
+        <v>107</v>
+      </c>
+      <c r="L15" t="s">
+        <v>17</v>
+      </c>
+      <c r="M15" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A16" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="B16" s="12" t="s">
+        <v>128</v>
+      </c>
+      <c r="C16" t="s">
+        <v>16</v>
+      </c>
+      <c r="D16" t="s">
+        <v>17</v>
+      </c>
+      <c r="E16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F16" t="s">
+        <v>17</v>
+      </c>
+      <c r="G16" t="s">
+        <v>17</v>
+      </c>
+      <c r="H16" t="s">
+        <v>110</v>
+      </c>
+      <c r="I16" t="s">
+        <v>17</v>
+      </c>
+      <c r="J16" t="s">
+        <v>17</v>
+      </c>
+      <c r="K16" t="s">
+        <v>107</v>
+      </c>
+      <c r="L16" t="s">
+        <v>17</v>
+      </c>
+      <c r="M16" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A17" s="12" t="s">
+        <v>129</v>
+      </c>
+      <c r="B17" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="C17" t="s">
+        <v>16</v>
+      </c>
+      <c r="D17" t="s">
+        <v>17</v>
+      </c>
+      <c r="E17" t="s">
+        <v>16</v>
+      </c>
+      <c r="F17" t="s">
+        <v>17</v>
+      </c>
+      <c r="G17" t="s">
+        <v>17</v>
+      </c>
+      <c r="H17" t="s">
+        <v>145</v>
+      </c>
+      <c r="I17" t="s">
+        <v>17</v>
+      </c>
+      <c r="J17" t="s">
+        <v>17</v>
+      </c>
+      <c r="K17" t="s">
+        <v>107</v>
+      </c>
+      <c r="L17" t="s">
+        <v>17</v>
+      </c>
+      <c r="M17" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A18" s="12" t="s">
+        <v>131</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>132</v>
+      </c>
+      <c r="C18" t="s">
+        <v>16</v>
+      </c>
+      <c r="D18" t="s">
+        <v>17</v>
+      </c>
+      <c r="E18" t="s">
+        <v>16</v>
+      </c>
+      <c r="F18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G18" t="s">
+        <v>17</v>
+      </c>
+      <c r="H18" t="s">
+        <v>110</v>
+      </c>
+      <c r="I18" t="s">
+        <v>17</v>
+      </c>
+      <c r="J18" t="s">
+        <v>17</v>
+      </c>
+      <c r="K18" t="s">
+        <v>107</v>
+      </c>
+      <c r="L18" t="s">
+        <v>17</v>
+      </c>
+      <c r="M18" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A19" s="12" t="s">
+        <v>133</v>
+      </c>
+      <c r="B19" s="12" t="s">
+        <v>134</v>
+      </c>
+      <c r="C19" t="s">
+        <v>16</v>
+      </c>
+      <c r="D19" t="s">
+        <v>17</v>
+      </c>
+      <c r="E19" t="s">
+        <v>16</v>
+      </c>
+      <c r="F19" t="s">
+        <v>17</v>
+      </c>
+      <c r="G19" t="s">
+        <v>17</v>
+      </c>
+      <c r="H19" t="s">
+        <v>110</v>
+      </c>
+      <c r="I19" t="s">
+        <v>17</v>
+      </c>
+      <c r="J19" t="s">
+        <v>17</v>
+      </c>
+      <c r="K19" t="s">
+        <v>107</v>
+      </c>
+      <c r="L19" t="s">
+        <v>17</v>
+      </c>
+      <c r="M19" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A20" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="B20" s="12" t="s">
+        <v>135</v>
+      </c>
+      <c r="C20" t="s">
+        <v>16</v>
+      </c>
+      <c r="D20" t="s">
+        <v>17</v>
+      </c>
+      <c r="E20" t="s">
+        <v>16</v>
+      </c>
+      <c r="F20" t="s">
+        <v>17</v>
+      </c>
+      <c r="G20" t="s">
+        <v>17</v>
+      </c>
+      <c r="H20" t="s">
+        <v>110</v>
+      </c>
+      <c r="I20" t="s">
+        <v>17</v>
+      </c>
+      <c r="J20" t="s">
+        <v>17</v>
+      </c>
+      <c r="K20" t="s">
+        <v>107</v>
+      </c>
+      <c r="L20" t="s">
+        <v>17</v>
+      </c>
+      <c r="M20" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A21" s="12" t="s">
+        <v>136</v>
+      </c>
+      <c r="B21" s="12" t="s">
+        <v>137</v>
+      </c>
+      <c r="C21" t="s">
+        <v>16</v>
+      </c>
+      <c r="D21" t="s">
+        <v>17</v>
+      </c>
+      <c r="E21" t="s">
+        <v>17</v>
+      </c>
+      <c r="F21" t="s">
+        <v>17</v>
+      </c>
+      <c r="G21" t="s">
+        <v>17</v>
+      </c>
+      <c r="H21" t="s">
+        <v>17</v>
+      </c>
+      <c r="I21" t="s">
+        <v>17</v>
+      </c>
+      <c r="J21" t="s">
+        <v>17</v>
+      </c>
+      <c r="K21" t="s">
+        <v>107</v>
+      </c>
+      <c r="L21" t="s">
+        <v>17</v>
+      </c>
+      <c r="M21" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A22" s="12" t="s">
+        <v>138</v>
+      </c>
+      <c r="B22" s="12" t="s">
+        <v>139</v>
+      </c>
+      <c r="C22" t="s">
+        <v>16</v>
+      </c>
+      <c r="D22" t="s">
+        <v>17</v>
+      </c>
+      <c r="E22" t="s">
+        <v>17</v>
+      </c>
+      <c r="F22" t="s">
+        <v>17</v>
+      </c>
+      <c r="G22" t="s">
+        <v>17</v>
+      </c>
+      <c r="H22" t="s">
+        <v>17</v>
+      </c>
+      <c r="I22" t="s">
+        <v>17</v>
+      </c>
+      <c r="J22" t="s">
+        <v>17</v>
+      </c>
+      <c r="K22" t="s">
+        <v>107</v>
+      </c>
+      <c r="L22" t="s">
+        <v>17</v>
+      </c>
+      <c r="M22" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A23" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="B23" s="12" t="s">
+        <v>140</v>
+      </c>
+      <c r="C23" t="s">
+        <v>16</v>
+      </c>
+      <c r="D23" t="s">
+        <v>16</v>
+      </c>
+      <c r="E23" t="s">
+        <v>17</v>
+      </c>
+      <c r="F23" t="s">
+        <v>143</v>
+      </c>
+      <c r="G23" t="s">
+        <v>146</v>
+      </c>
+      <c r="H23" t="s">
+        <v>110</v>
+      </c>
+      <c r="I23" t="s">
+        <v>17</v>
+      </c>
+      <c r="J23" t="s">
+        <v>17</v>
+      </c>
+      <c r="K23" t="s">
+        <v>107</v>
+      </c>
+      <c r="L23" t="s">
+        <v>17</v>
+      </c>
+      <c r="M23" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A24" s="12" t="s">
+        <v>141</v>
+      </c>
+      <c r="B24" s="12" t="s">
+        <v>142</v>
+      </c>
+      <c r="C24" t="s">
+        <v>16</v>
+      </c>
+      <c r="D24" t="s">
+        <v>17</v>
+      </c>
+      <c r="E24" t="s">
+        <v>17</v>
+      </c>
+      <c r="F24" t="s">
+        <v>17</v>
+      </c>
+      <c r="G24" t="s">
+        <v>17</v>
+      </c>
+      <c r="H24" t="s">
+        <v>17</v>
+      </c>
+      <c r="I24" t="s">
+        <v>17</v>
+      </c>
+      <c r="J24" t="s">
+        <v>17</v>
+      </c>
+      <c r="K24" t="s">
+        <v>107</v>
+      </c>
+      <c r="L24" t="s">
+        <v>17</v>
+      </c>
+      <c r="M24" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A25" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="B25" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="C25" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25" t="s">
+        <v>17</v>
+      </c>
+      <c r="E25" t="s">
+        <v>17</v>
+      </c>
+      <c r="F25" t="s">
+        <v>17</v>
+      </c>
+      <c r="G25" t="s">
+        <v>17</v>
+      </c>
+      <c r="H25" t="s">
+        <v>110</v>
+      </c>
+      <c r="I25" t="s">
+        <v>17</v>
+      </c>
+      <c r="J25" t="s">
+        <v>17</v>
+      </c>
+      <c r="K25" t="s">
+        <v>107</v>
+      </c>
+      <c r="L25" t="s">
+        <v>17</v>
+      </c>
+      <c r="M25" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A26" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="B26" s="10" t="s">
+        <v>87</v>
+      </c>
+      <c r="C26" t="s">
+        <v>16</v>
+      </c>
+      <c r="D26" t="s">
+        <v>17</v>
+      </c>
+      <c r="E26" t="s">
+        <v>16</v>
+      </c>
+      <c r="F26" t="s">
+        <v>17</v>
+      </c>
+      <c r="G26" t="s">
+        <v>17</v>
+      </c>
+      <c r="H26" t="s">
+        <v>145</v>
+      </c>
+      <c r="I26" t="s">
+        <v>17</v>
+      </c>
+      <c r="J26" t="s">
+        <v>17</v>
+      </c>
+      <c r="K26" t="s">
+        <v>107</v>
+      </c>
+      <c r="L26" t="s">
+        <v>17</v>
+      </c>
+      <c r="M26" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A27" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="B27" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="C27" t="s">
+        <v>16</v>
+      </c>
+      <c r="D27" t="s">
+        <v>17</v>
+      </c>
+      <c r="E27" t="s">
+        <v>16</v>
+      </c>
+      <c r="F27" t="s">
+        <v>17</v>
+      </c>
+      <c r="G27" t="s">
+        <v>17</v>
+      </c>
+      <c r="H27" t="s">
+        <v>110</v>
+      </c>
+      <c r="I27" t="s">
+        <v>17</v>
+      </c>
+      <c r="J27" t="s">
+        <v>17</v>
+      </c>
+      <c r="K27" t="s">
+        <v>107</v>
+      </c>
+      <c r="L27" t="s">
+        <v>17</v>
+      </c>
+      <c r="M27" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A28" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="B28" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="C28" t="s">
+        <v>16</v>
+      </c>
+      <c r="D28" t="s">
+        <v>17</v>
+      </c>
+      <c r="E28" t="s">
+        <v>16</v>
+      </c>
+      <c r="F28" t="s">
+        <v>17</v>
+      </c>
+      <c r="G28" t="s">
+        <v>17</v>
+      </c>
+      <c r="H28" t="s">
+        <v>110</v>
+      </c>
+      <c r="I28" t="s">
+        <v>17</v>
+      </c>
+      <c r="J28" t="s">
+        <v>17</v>
+      </c>
+      <c r="K28" t="s">
+        <v>107</v>
+      </c>
+      <c r="L28" t="s">
+        <v>17</v>
+      </c>
+      <c r="M28" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A29" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="B29" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="C29" t="s">
+        <v>16</v>
+      </c>
+      <c r="D29" t="s">
+        <v>17</v>
+      </c>
+      <c r="E29" t="s">
+        <v>16</v>
+      </c>
+      <c r="F29" t="s">
+        <v>17</v>
+      </c>
+      <c r="G29" t="s">
+        <v>17</v>
+      </c>
+      <c r="H29" t="s">
+        <v>110</v>
+      </c>
+      <c r="I29" t="s">
+        <v>17</v>
+      </c>
+      <c r="J29" t="s">
+        <v>17</v>
+      </c>
+      <c r="K29" t="s">
+        <v>107</v>
+      </c>
+      <c r="L29" t="s">
+        <v>17</v>
+      </c>
+      <c r="M29" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A30" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B30" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="C30" t="s">
+        <v>16</v>
+      </c>
+      <c r="D30" t="s">
+        <v>17</v>
+      </c>
+      <c r="E30" t="s">
+        <v>17</v>
+      </c>
+      <c r="F30" t="s">
+        <v>17</v>
+      </c>
+      <c r="G30" t="s">
+        <v>17</v>
+      </c>
+      <c r="H30" t="s">
+        <v>17</v>
+      </c>
+      <c r="I30" t="s">
+        <v>17</v>
+      </c>
+      <c r="J30" t="s">
+        <v>17</v>
+      </c>
+      <c r="K30" t="s">
+        <v>107</v>
+      </c>
+      <c r="L30" t="s">
+        <v>17</v>
+      </c>
+      <c r="M30" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A31" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="B31" s="10" t="s">
+        <v>97</v>
+      </c>
+      <c r="C31" t="s">
+        <v>16</v>
+      </c>
+      <c r="D31" t="s">
+        <v>17</v>
+      </c>
+      <c r="E31" t="s">
+        <v>17</v>
+      </c>
+      <c r="F31" t="s">
+        <v>17</v>
+      </c>
+      <c r="G31" t="s">
+        <v>17</v>
+      </c>
+      <c r="H31" t="s">
+        <v>17</v>
+      </c>
+      <c r="I31" t="s">
+        <v>17</v>
+      </c>
+      <c r="J31" t="s">
+        <v>17</v>
+      </c>
+      <c r="K31" t="s">
+        <v>107</v>
+      </c>
+      <c r="L31" t="s">
+        <v>17</v>
+      </c>
+      <c r="M31" t="s">
+        <v>16</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:M31" xr:uid="{928F2DD2-5FFA-4840-99B4-B7403ECB3D45}"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="22.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>